<commit_message>
updated pooled counts dataset
</commit_message>
<xml_diff>
--- a/LOT2_pooled_counts.xlsx
+++ b/LOT2_pooled_counts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valeriehofstetter/Desktop/LoT2_PAPER/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valeriehofstetter/Desktop/LoT2_PAPER/MANUSCRIPT/RESULTATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2DF46F-1256-3E48-A3A4-924344AF4FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D80D96B8-91B7-AD46-8DF3-DED88ADFB47D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="600" windowWidth="32420" windowHeight="20200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="620" windowWidth="28380" windowHeight="19680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL isolates" sheetId="5" r:id="rId1"/>
@@ -7427,7 +7427,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7510,8 +7510,15 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7638,6 +7645,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -7705,7 +7718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -8115,6 +8128,12 @@
     <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15439,8 +15458,8 @@
       <c r="B160" s="9" t="s">
         <v>1914</v>
       </c>
-      <c r="C160" s="130">
-        <v>1</v>
+      <c r="C160" s="138">
+        <v>2</v>
       </c>
       <c r="D160" s="18">
         <v>0</v>
@@ -15477,14 +15496,14 @@
       </c>
     </row>
     <row r="161" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="108">
-        <v>104</v>
+      <c r="A161" s="137">
+        <v>105</v>
       </c>
       <c r="B161" s="9" t="s">
         <v>2001</v>
       </c>
-      <c r="C161" s="130">
-        <v>7</v>
+      <c r="C161" s="138">
+        <v>6</v>
       </c>
       <c r="D161" s="18">
         <v>0</v>

</xml_diff>